<commit_message>
feat: add lesson for adding borders to cells in a spreadsheet
</commit_message>
<xml_diff>
--- a/styles.xlsx
+++ b/styles.xlsx
@@ -48,7 +48,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -56,15 +56,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="00000000"/>
+      </left>
+      <right style="double">
+        <color rgb="00000000"/>
+      </right>
+      <top style="double">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="double">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="double">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,7 +496,7 @@
           <t>April</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Purple</t>
         </is>

</xml_diff>